<commit_message>
Se añadió modal para importar listado de activos fijos en excel
</commit_message>
<xml_diff>
--- a/ERPSEI/wwwroot/templates/PlantillaActivosFijos.xlsx
+++ b/ERPSEI/wwwroot/templates/PlantillaActivosFijos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge Cruz\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D643EAF9-B72C-4001-9A51-20365CF6D7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE0532C-68CF-4A37-A510-6BC78A77E574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>Id</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Folio</t>
   </si>
@@ -34,9 +31,6 @@
     <t>Responsable</t>
   </si>
   <si>
-    <t>Categoría</t>
-  </si>
-  <si>
     <t>Tipo</t>
   </si>
   <si>
@@ -56,6 +50,18 @@
   </si>
   <si>
     <t>Comentarios</t>
+  </si>
+  <si>
+    <t>Marca</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Fecha Renovación</t>
+  </si>
+  <si>
+    <t>Deshabilitado</t>
   </si>
 </sst>
 </file>
@@ -116,12 +122,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,158 +461,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.44140625" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="20.6640625" customWidth="1"/>
+    <col min="12" max="12" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>